<commit_message>
add testlink docx generated and the diagram for the excel file
</commit_message>
<xml_diff>
--- a/docs/Lab03/Lab03_WBT_TCs_Form.xlsx
+++ b/docs/Lab03/Lab03_WBT_TCs_Form.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E257804-A6C6-4C1A-B702-6E76BE861F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3D3911-A48E-49A0-AA3A-7D85AA7ABE53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Statement" sheetId="1" r:id="rId1"/>
@@ -33,8 +33,40 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="2">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="2">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="140">
   <si>
     <t>VVSS, Info Romana, 2025-2026</t>
   </si>
@@ -100,9 +132,6 @@
   </si>
   <si>
     <t>Req02_L02</t>
-  </si>
-  <si>
-    <t>&lt;Req02 CFG &gt;</t>
   </si>
   <si>
     <t>CC3 = No. of Conditions + 1 =</t>
@@ -1347,7 +1376,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1431,210 +1460,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1651,48 +1476,251 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1756,80 +1784,6 @@
         <a:xfrm>
           <a:off x="567690" y="1208662"/>
           <a:ext cx="4381284" cy="2363497"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>621030</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>125730</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>194310</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>101847</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6188" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-00002C180000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="5208270" y="1588770"/>
-          <a:ext cx="4724400" cy="4168140"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2392,6 +2346,75 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+</richValueRels>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -2743,7 +2766,7 @@
         <v>9</v>
       </c>
       <c r="O7" s="26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P7" s="26">
         <v>237</v>
@@ -2758,7 +2781,7 @@
         <v>10</v>
       </c>
       <c r="O8" s="26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="P8" s="26">
         <v>237</v>
@@ -2779,7 +2802,7 @@
     </row>
     <row r="11" spans="2:16">
       <c r="B11" s="36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -2830,18 +2853,18 @@
       <c r="I1" s="65"/>
     </row>
     <row r="3" spans="2:20">
-      <c r="B3" s="103" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="83"/>
+      <c r="B3" s="100" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="102"/>
     </row>
     <row r="6" spans="2:20">
       <c r="B6" s="63" t="s">
@@ -2872,21 +2895,21 @@
       <c r="B8" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="93" t="s">
+      <c r="C8" s="114" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
+      <c r="D8" s="114"/>
+      <c r="E8" s="114"/>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
       <c r="I8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="Q8" s="81" t="s">
+      <c r="Q8" s="113" t="s">
         <v>17</v>
       </c>
-      <c r="R8" s="81"/>
-      <c r="S8" s="81"/>
+      <c r="R8" s="113"/>
+      <c r="S8" s="113"/>
       <c r="T8" s="33">
         <v>6</v>
       </c>
@@ -2895,112 +2918,115 @@
       <c r="B9" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="80" t="s">
+      <c r="C9" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="80"/>
-      <c r="E9" s="80"/>
+      <c r="D9" s="103"/>
+      <c r="E9" s="103"/>
       <c r="F9" s="35"/>
       <c r="G9" s="35"/>
+      <c r="H9" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="I9" s="37"/>
-      <c r="Q9" s="81" t="s">
+      <c r="Q9" s="113" t="s">
         <v>20</v>
       </c>
-      <c r="R9" s="81"/>
-      <c r="S9" s="81"/>
+      <c r="R9" s="113"/>
+      <c r="S9" s="113"/>
       <c r="T9" s="33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="2:20">
       <c r="B10" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="80" t="s">
+      <c r="C10" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="80"/>
-      <c r="E10" s="80"/>
+      <c r="D10" s="103"/>
+      <c r="E10" s="103"/>
       <c r="F10" s="35"/>
       <c r="G10" s="35"/>
-      <c r="I10" s="84" t="s">
+      <c r="I10" s="104" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="J10" s="105"/>
+      <c r="K10" s="105"/>
+      <c r="L10" s="105"/>
+      <c r="M10" s="105"/>
+      <c r="N10" s="105"/>
+      <c r="O10" s="106"/>
+      <c r="Q10" s="113" t="s">
         <v>22</v>
       </c>
-      <c r="J10" s="85"/>
-      <c r="K10" s="85"/>
-      <c r="L10" s="85"/>
-      <c r="M10" s="85"/>
-      <c r="N10" s="85"/>
-      <c r="O10" s="86"/>
-      <c r="Q10" s="81" t="s">
+      <c r="R10" s="113" t="s">
         <v>23</v>
       </c>
-      <c r="R10" s="81" t="s">
-        <v>24</v>
-      </c>
-      <c r="S10" s="81"/>
+      <c r="S10" s="113"/>
       <c r="T10" s="33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="2:20">
       <c r="B11" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="80" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="80"/>
-      <c r="E11" s="80"/>
+      <c r="D11" s="103"/>
+      <c r="E11" s="103"/>
       <c r="F11" s="35"/>
       <c r="G11" s="35"/>
-      <c r="I11" s="87"/>
-      <c r="J11" s="88"/>
-      <c r="K11" s="88"/>
-      <c r="L11" s="88"/>
-      <c r="M11" s="88"/>
-      <c r="N11" s="88"/>
-      <c r="O11" s="89"/>
+      <c r="I11" s="107"/>
+      <c r="J11" s="108"/>
+      <c r="K11" s="108"/>
+      <c r="L11" s="108"/>
+      <c r="M11" s="108"/>
+      <c r="N11" s="108"/>
+      <c r="O11" s="109"/>
     </row>
     <row r="12" spans="2:20">
       <c r="B12" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="80" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="80"/>
-      <c r="E12" s="80"/>
+      <c r="D12" s="103"/>
+      <c r="E12" s="103"/>
       <c r="F12" s="35"/>
       <c r="G12" s="35"/>
-      <c r="I12" s="87"/>
-      <c r="J12" s="88"/>
-      <c r="K12" s="88"/>
-      <c r="L12" s="88"/>
-      <c r="M12" s="88"/>
-      <c r="N12" s="88"/>
-      <c r="O12" s="89"/>
+      <c r="I12" s="107"/>
+      <c r="J12" s="108"/>
+      <c r="K12" s="108"/>
+      <c r="L12" s="108"/>
+      <c r="M12" s="108"/>
+      <c r="N12" s="108"/>
+      <c r="O12" s="109"/>
     </row>
     <row r="13" spans="2:20">
       <c r="B13" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="80" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="80"/>
-      <c r="E13" s="80"/>
+      <c r="D13" s="103"/>
+      <c r="E13" s="103"/>
       <c r="F13" s="35"/>
       <c r="G13" s="35"/>
-      <c r="I13" s="87"/>
-      <c r="J13" s="88"/>
-      <c r="K13" s="88"/>
-      <c r="L13" s="88"/>
-      <c r="M13" s="88"/>
-      <c r="N13" s="88"/>
-      <c r="O13" s="89"/>
+      <c r="I13" s="107"/>
+      <c r="J13" s="108"/>
+      <c r="K13" s="108"/>
+      <c r="L13" s="108"/>
+      <c r="M13" s="108"/>
+      <c r="N13" s="108"/>
+      <c r="O13" s="109"/>
       <c r="Q13" s="63" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R13" s="64"/>
       <c r="S13" s="64"/>
@@ -3008,171 +3034,179 @@
     </row>
     <row r="14" spans="2:20">
       <c r="B14" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="80" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="80"/>
-      <c r="E14" s="80"/>
+      <c r="D14" s="103"/>
+      <c r="E14" s="103"/>
       <c r="F14" s="35"/>
       <c r="G14" s="35"/>
-      <c r="I14" s="87"/>
-      <c r="J14" s="88"/>
-      <c r="K14" s="88"/>
-      <c r="L14" s="88"/>
-      <c r="M14" s="88"/>
-      <c r="N14" s="88"/>
-      <c r="O14" s="89"/>
+      <c r="I14" s="107"/>
+      <c r="J14" s="108"/>
+      <c r="K14" s="108"/>
+      <c r="L14" s="108"/>
+      <c r="M14" s="108"/>
+      <c r="N14" s="108"/>
+      <c r="O14" s="109"/>
     </row>
     <row r="15" spans="2:20">
-      <c r="I15" s="87"/>
-      <c r="J15" s="88"/>
-      <c r="K15" s="88"/>
-      <c r="L15" s="88"/>
-      <c r="M15" s="88"/>
-      <c r="N15" s="88"/>
-      <c r="O15" s="89"/>
+      <c r="I15" s="107"/>
+      <c r="J15" s="108"/>
+      <c r="K15" s="108"/>
+      <c r="L15" s="108"/>
+      <c r="M15" s="108"/>
+      <c r="N15" s="108"/>
+      <c r="O15" s="109"/>
       <c r="Q15" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="R15" s="114" t="s">
         <v>29</v>
       </c>
-      <c r="R15" s="93" t="s">
+      <c r="S15" s="114"/>
+      <c r="T15" s="114"/>
+    </row>
+    <row r="16" spans="2:20">
+      <c r="I16" s="107"/>
+      <c r="J16" s="108"/>
+      <c r="K16" s="108"/>
+      <c r="L16" s="108"/>
+      <c r="M16" s="108"/>
+      <c r="N16" s="108"/>
+      <c r="O16" s="109"/>
+      <c r="Q16" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="S15" s="93"/>
-      <c r="T15" s="93"/>
-    </row>
-    <row r="16" spans="2:20">
-      <c r="I16" s="87"/>
-      <c r="J16" s="88"/>
-      <c r="K16" s="88"/>
-      <c r="L16" s="88"/>
-      <c r="M16" s="88"/>
-      <c r="N16" s="88"/>
-      <c r="O16" s="89"/>
-      <c r="Q16" s="34" t="s">
+      <c r="R16" s="99" t="s">
+        <v>81</v>
+      </c>
+      <c r="S16" s="99"/>
+      <c r="T16" s="99"/>
+    </row>
+    <row r="17" spans="9:20">
+      <c r="I17" s="107"/>
+      <c r="J17" s="108"/>
+      <c r="K17" s="108"/>
+      <c r="L17" s="108"/>
+      <c r="M17" s="108"/>
+      <c r="N17" s="108"/>
+      <c r="O17" s="109"/>
+      <c r="Q17" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="R16" s="79" t="s">
+      <c r="R17" s="99" t="s">
         <v>82</v>
       </c>
-      <c r="S16" s="79"/>
-      <c r="T16" s="79"/>
-    </row>
-    <row r="17" spans="9:20">
-      <c r="I17" s="87"/>
-      <c r="J17" s="88"/>
-      <c r="K17" s="88"/>
-      <c r="L17" s="88"/>
-      <c r="M17" s="88"/>
-      <c r="N17" s="88"/>
-      <c r="O17" s="89"/>
-      <c r="Q17" s="34" t="s">
+      <c r="S17" s="99"/>
+      <c r="T17" s="99"/>
+    </row>
+    <row r="18" spans="9:20" ht="12.75" customHeight="1">
+      <c r="I18" s="107"/>
+      <c r="J18" s="108"/>
+      <c r="K18" s="108"/>
+      <c r="L18" s="108"/>
+      <c r="M18" s="108"/>
+      <c r="N18" s="108"/>
+      <c r="O18" s="109"/>
+      <c r="Q18" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="R17" s="79" t="s">
+      <c r="R18" s="115" t="s">
         <v>83</v>
       </c>
-      <c r="S17" s="79"/>
-      <c r="T17" s="79"/>
-    </row>
-    <row r="18" spans="9:20" ht="12.75" customHeight="1">
-      <c r="I18" s="87"/>
-      <c r="J18" s="88"/>
-      <c r="K18" s="88"/>
-      <c r="L18" s="88"/>
-      <c r="M18" s="88"/>
-      <c r="N18" s="88"/>
-      <c r="O18" s="89"/>
-      <c r="Q18" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="R18" s="104" t="s">
+      <c r="S18" s="116"/>
+      <c r="T18" s="117"/>
+    </row>
+    <row r="19" spans="9:20">
+      <c r="I19" s="107"/>
+      <c r="J19" s="108"/>
+      <c r="K19" s="108"/>
+      <c r="L19" s="108"/>
+      <c r="M19" s="108"/>
+      <c r="N19" s="108"/>
+      <c r="O19" s="109"/>
+      <c r="Q19" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="R19" s="99" t="s">
         <v>84</v>
       </c>
-      <c r="S18" s="105"/>
-      <c r="T18" s="106"/>
-    </row>
-    <row r="19" spans="9:20">
-      <c r="I19" s="87"/>
-      <c r="J19" s="88"/>
-      <c r="K19" s="88"/>
-      <c r="L19" s="88"/>
-      <c r="M19" s="88"/>
-      <c r="N19" s="88"/>
-      <c r="O19" s="89"/>
-      <c r="Q19" s="34" t="s">
+      <c r="S19" s="99"/>
+      <c r="T19" s="99"/>
+    </row>
+    <row r="20" spans="9:20">
+      <c r="I20" s="107"/>
+      <c r="J20" s="108"/>
+      <c r="K20" s="108"/>
+      <c r="L20" s="108"/>
+      <c r="M20" s="108"/>
+      <c r="N20" s="108"/>
+      <c r="O20" s="109"/>
+      <c r="Q20" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="R19" s="79" t="s">
-        <v>85</v>
-      </c>
-      <c r="S19" s="79"/>
-      <c r="T19" s="79"/>
-    </row>
-    <row r="20" spans="9:20">
-      <c r="I20" s="87"/>
-      <c r="J20" s="88"/>
-      <c r="K20" s="88"/>
-      <c r="L20" s="88"/>
-      <c r="M20" s="88"/>
-      <c r="N20" s="88"/>
-      <c r="O20" s="89"/>
-      <c r="Q20" s="34" t="s">
+      <c r="R20" s="99" t="s">
+        <v>88</v>
+      </c>
+      <c r="S20" s="99"/>
+      <c r="T20" s="99"/>
+    </row>
+    <row r="21" spans="9:20">
+      <c r="I21" s="107"/>
+      <c r="J21" s="108"/>
+      <c r="K21" s="108"/>
+      <c r="L21" s="108"/>
+      <c r="M21" s="108"/>
+      <c r="N21" s="108"/>
+      <c r="O21" s="109"/>
+      <c r="Q21" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="R20" s="79" t="s">
+      <c r="R21" s="99" t="s">
         <v>89</v>
       </c>
-      <c r="S20" s="79"/>
-      <c r="T20" s="79"/>
-    </row>
-    <row r="21" spans="9:20">
-      <c r="I21" s="87"/>
-      <c r="J21" s="88"/>
-      <c r="K21" s="88"/>
-      <c r="L21" s="88"/>
-      <c r="M21" s="88"/>
-      <c r="N21" s="88"/>
-      <c r="O21" s="89"/>
-      <c r="Q21" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="R21" s="79" t="s">
-        <v>90</v>
-      </c>
-      <c r="S21" s="79"/>
-      <c r="T21" s="79"/>
+      <c r="S21" s="99"/>
+      <c r="T21" s="99"/>
     </row>
     <row r="22" spans="9:20">
-      <c r="I22" s="87"/>
-      <c r="J22" s="88"/>
-      <c r="K22" s="88"/>
-      <c r="L22" s="88"/>
-      <c r="M22" s="88"/>
-      <c r="N22" s="88"/>
-      <c r="O22" s="89"/>
+      <c r="I22" s="107"/>
+      <c r="J22" s="108"/>
+      <c r="K22" s="108"/>
+      <c r="L22" s="108"/>
+      <c r="M22" s="108"/>
+      <c r="N22" s="108"/>
+      <c r="O22" s="109"/>
     </row>
     <row r="23" spans="9:20">
-      <c r="I23" s="87"/>
-      <c r="J23" s="88"/>
-      <c r="K23" s="88"/>
-      <c r="L23" s="88"/>
-      <c r="M23" s="88"/>
-      <c r="N23" s="88"/>
-      <c r="O23" s="89"/>
+      <c r="I23" s="107"/>
+      <c r="J23" s="108"/>
+      <c r="K23" s="108"/>
+      <c r="L23" s="108"/>
+      <c r="M23" s="108"/>
+      <c r="N23" s="108"/>
+      <c r="O23" s="109"/>
     </row>
     <row r="24" spans="9:20">
-      <c r="I24" s="90"/>
-      <c r="J24" s="91"/>
-      <c r="K24" s="91"/>
-      <c r="L24" s="91"/>
-      <c r="M24" s="91"/>
-      <c r="N24" s="91"/>
-      <c r="O24" s="92"/>
+      <c r="I24" s="110"/>
+      <c r="J24" s="111"/>
+      <c r="K24" s="111"/>
+      <c r="L24" s="111"/>
+      <c r="M24" s="111"/>
+      <c r="N24" s="111"/>
+      <c r="O24" s="112"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="R18:T18"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="Q13:T13"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="R20:T20"/>
     <mergeCell ref="R21:T21"/>
@@ -3189,14 +3223,6 @@
     <mergeCell ref="Q6:T6"/>
     <mergeCell ref="R17:T17"/>
     <mergeCell ref="R19:T19"/>
-    <mergeCell ref="R18:T18"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="Q9:S9"/>
-    <mergeCell ref="R16:T16"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="Q13:T13"/>
-    <mergeCell ref="C14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3241,234 +3267,234 @@
       <c r="G1" s="65"/>
     </row>
     <row r="3" spans="2:26">
-      <c r="B3" s="103" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="83"/>
+      <c r="B3" s="100" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="102"/>
     </row>
     <row r="5" spans="2:26">
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="2:26" ht="15.75">
-      <c r="B6" s="100" t="s">
+      <c r="B6" s="118" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="118" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="100" t="s">
+      <c r="D6" s="119" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="101" t="s">
+      <c r="E6" s="118" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="100" t="s">
+      <c r="F6" s="118"/>
+      <c r="G6" s="118"/>
+      <c r="H6" s="118"/>
+      <c r="I6" s="118"/>
+      <c r="J6" s="118"/>
+      <c r="K6" s="118"/>
+      <c r="L6" s="118"/>
+      <c r="M6" s="118"/>
+      <c r="N6" s="118"/>
+      <c r="O6" s="118"/>
+      <c r="P6" s="118"/>
+      <c r="Q6" s="118"/>
+      <c r="R6" s="118"/>
+      <c r="S6" s="118"/>
+      <c r="T6" s="118"/>
+      <c r="U6" s="118"/>
+      <c r="V6" s="118"/>
+      <c r="W6" s="118"/>
+      <c r="X6" s="118"/>
+      <c r="Y6" s="118"/>
+      <c r="Z6" s="118"/>
+    </row>
+    <row r="7" spans="2:26" ht="15.75">
+      <c r="B7" s="118"/>
+      <c r="C7" s="118"/>
+      <c r="D7" s="120"/>
+      <c r="E7" s="126" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="100"/>
-      <c r="G6" s="100"/>
-      <c r="H6" s="100"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="100"/>
-      <c r="K6" s="100"/>
-      <c r="L6" s="100"/>
-      <c r="M6" s="100"/>
-      <c r="N6" s="100"/>
-      <c r="O6" s="100"/>
-      <c r="P6" s="100"/>
-      <c r="Q6" s="100"/>
-      <c r="R6" s="100"/>
-      <c r="S6" s="100"/>
-      <c r="T6" s="100"/>
-      <c r="U6" s="100"/>
-      <c r="V6" s="100"/>
-      <c r="W6" s="100"/>
-      <c r="X6" s="100"/>
-      <c r="Y6" s="100"/>
-      <c r="Z6" s="100"/>
-    </row>
-    <row r="7" spans="2:26" ht="15.75">
-      <c r="B7" s="100"/>
-      <c r="C7" s="100"/>
-      <c r="D7" s="102"/>
-      <c r="E7" s="97" t="s">
+      <c r="F7" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="96" t="s">
+      <c r="G7" s="125"/>
+      <c r="H7" s="125"/>
+      <c r="I7" s="125"/>
+      <c r="J7" s="125"/>
+      <c r="K7" s="125"/>
+      <c r="L7" s="125"/>
+      <c r="M7" s="125"/>
+      <c r="N7" s="122" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="96"/>
-      <c r="H7" s="96"/>
-      <c r="I7" s="96"/>
-      <c r="J7" s="96"/>
-      <c r="K7" s="96"/>
-      <c r="L7" s="96"/>
-      <c r="M7" s="96"/>
-      <c r="N7" s="98" t="s">
+      <c r="O7" s="122"/>
+      <c r="P7" s="122"/>
+      <c r="Q7" s="122"/>
+      <c r="R7" s="122"/>
+      <c r="S7" s="122"/>
+      <c r="T7" s="121" t="s">
         <v>40</v>
       </c>
-      <c r="O7" s="98"/>
-      <c r="P7" s="98"/>
-      <c r="Q7" s="98"/>
-      <c r="R7" s="98"/>
-      <c r="S7" s="98"/>
-      <c r="T7" s="99" t="s">
+      <c r="U7" s="121"/>
+      <c r="V7" s="121"/>
+      <c r="W7" s="121"/>
+      <c r="X7" s="121"/>
+      <c r="Y7" s="121"/>
+      <c r="Z7" s="121"/>
+    </row>
+    <row r="8" spans="2:26" ht="15.6" customHeight="1">
+      <c r="B8" s="118"/>
+      <c r="C8" s="123" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="123" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="126"/>
+      <c r="F8" s="125" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="125"/>
+      <c r="H8" s="125" t="s">
+        <v>91</v>
+      </c>
+      <c r="I8" s="125"/>
+      <c r="J8" s="125" t="s">
+        <v>92</v>
+      </c>
+      <c r="K8" s="125"/>
+      <c r="L8" s="125" t="s">
+        <v>93</v>
+      </c>
+      <c r="M8" s="125"/>
+      <c r="N8" s="122" t="s">
+        <v>30</v>
+      </c>
+      <c r="O8" s="122" t="s">
+        <v>31</v>
+      </c>
+      <c r="P8" s="122" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q8" s="122" t="s">
+        <v>85</v>
+      </c>
+      <c r="R8" s="122" t="s">
+        <v>86</v>
+      </c>
+      <c r="S8" s="122" t="s">
+        <v>87</v>
+      </c>
+      <c r="T8" s="121">
+        <v>0</v>
+      </c>
+      <c r="U8" s="121">
+        <v>1</v>
+      </c>
+      <c r="V8" s="121">
+        <v>2</v>
+      </c>
+      <c r="W8" s="121" t="s">
         <v>41</v>
       </c>
-      <c r="U7" s="99"/>
-      <c r="V7" s="99"/>
-      <c r="W7" s="99"/>
-      <c r="X7" s="99"/>
-      <c r="Y7" s="99"/>
-      <c r="Z7" s="99"/>
-    </row>
-    <row r="8" spans="2:26" ht="15.6" customHeight="1">
-      <c r="B8" s="100"/>
-      <c r="C8" s="94" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="94" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="97"/>
-      <c r="F8" s="96" t="s">
-        <v>91</v>
-      </c>
-      <c r="G8" s="96"/>
-      <c r="H8" s="96" t="s">
-        <v>92</v>
-      </c>
-      <c r="I8" s="96"/>
-      <c r="J8" s="96" t="s">
-        <v>93</v>
-      </c>
-      <c r="K8" s="96"/>
-      <c r="L8" s="96" t="s">
-        <v>94</v>
-      </c>
-      <c r="M8" s="96"/>
-      <c r="N8" s="98" t="s">
-        <v>31</v>
-      </c>
-      <c r="O8" s="98" t="s">
-        <v>32</v>
-      </c>
-      <c r="P8" s="98" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" s="98" t="s">
-        <v>86</v>
-      </c>
-      <c r="R8" s="98" t="s">
-        <v>87</v>
-      </c>
-      <c r="S8" s="98" t="s">
-        <v>88</v>
-      </c>
-      <c r="T8" s="99">
-        <v>0</v>
-      </c>
-      <c r="U8" s="99">
-        <v>1</v>
-      </c>
-      <c r="V8" s="99">
-        <v>2</v>
-      </c>
-      <c r="W8" s="99" t="s">
+      <c r="X8" s="121" t="s">
         <v>42</v>
       </c>
-      <c r="X8" s="99" t="s">
+      <c r="Y8" s="121" t="s">
         <v>43</v>
       </c>
-      <c r="Y8" s="99" t="s">
+      <c r="Z8" s="121" t="s">
         <v>44</v>
       </c>
-      <c r="Z8" s="99" t="s">
+    </row>
+    <row r="9" spans="2:26" ht="15.75">
+      <c r="B9" s="118"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="124"/>
+      <c r="E9" s="126"/>
+      <c r="F9" s="13" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="2:26" ht="15.75">
-      <c r="B9" s="100"/>
-      <c r="C9" s="95"/>
-      <c r="D9" s="95"/>
-      <c r="E9" s="97"/>
-      <c r="F9" s="13" t="s">
+      <c r="G9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>47</v>
-      </c>
       <c r="H9" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="I9" s="13" t="s">
-        <v>47</v>
-      </c>
       <c r="J9" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="K9" s="13" t="s">
-        <v>47</v>
-      </c>
       <c r="L9" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="M9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="M9" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="N9" s="98"/>
-      <c r="O9" s="98"/>
-      <c r="P9" s="98"/>
-      <c r="Q9" s="98"/>
-      <c r="R9" s="98"/>
-      <c r="S9" s="98"/>
-      <c r="T9" s="99"/>
-      <c r="U9" s="99"/>
-      <c r="V9" s="99"/>
-      <c r="W9" s="99"/>
-      <c r="X9" s="99"/>
-      <c r="Y9" s="99"/>
-      <c r="Z9" s="99"/>
+      <c r="N9" s="122"/>
+      <c r="O9" s="122"/>
+      <c r="P9" s="122"/>
+      <c r="Q9" s="122"/>
+      <c r="R9" s="122"/>
+      <c r="S9" s="122"/>
+      <c r="T9" s="121"/>
+      <c r="U9" s="121"/>
+      <c r="V9" s="121"/>
+      <c r="W9" s="121"/>
+      <c r="X9" s="121"/>
+      <c r="Y9" s="121"/>
+      <c r="Z9" s="121"/>
     </row>
     <row r="10" spans="2:26" ht="15.75">
       <c r="B10" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="E10" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="F10" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="F10" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="G10" s="17" t="s">
+      <c r="H10" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="J10" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="L10" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="M10" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10" s="18" t="s">
         <v>98</v>
-      </c>
-      <c r="H10" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="I10" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="J10" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="K10" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="L10" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="M10" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="N10" s="18" t="s">
-        <v>99</v>
       </c>
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
@@ -3487,44 +3513,44 @@
     </row>
     <row r="11" spans="2:26" ht="15.75">
       <c r="B11" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="E11" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>102</v>
-      </c>
       <c r="F11" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I11" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J11" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K11" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L11" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M11" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N11" s="18"/>
       <c r="O11" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P11" s="18"/>
       <c r="Q11" s="18"/>
@@ -3542,45 +3568,45 @@
     </row>
     <row r="12" spans="2:26" ht="15.75">
       <c r="B12" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="C12" s="108" t="s">
+        <v>103</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="41" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="109" t="s">
-        <v>101</v>
-      </c>
-      <c r="E12" s="110" t="s">
-        <v>109</v>
-      </c>
       <c r="F12" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J12" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L12" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M12" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N12" s="18"/>
       <c r="O12" s="18"/>
       <c r="P12" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q12" s="18"/>
       <c r="R12" s="18"/>
@@ -3597,46 +3623,46 @@
     </row>
     <row r="13" spans="2:26" ht="15.75">
       <c r="B13" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C13" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" s="39" t="s">
         <v>114</v>
       </c>
-      <c r="D13" s="107" t="s">
+      <c r="E13" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="E13" s="16" t="s">
-        <v>116</v>
-      </c>
       <c r="F13" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H13" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="J13" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="K13" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="I13" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="J13" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="K13" s="17" t="s">
-        <v>47</v>
-      </c>
       <c r="L13" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M13" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N13" s="18"/>
       <c r="O13" s="18"/>
       <c r="P13" s="18"/>
       <c r="Q13" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="R13" s="18"/>
       <c r="S13" s="18"/>
@@ -3652,47 +3678,47 @@
     </row>
     <row r="14" spans="2:26" ht="15.75">
       <c r="B14" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C14" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
         <v>117</v>
       </c>
-      <c r="D14" t="s">
-        <v>118</v>
-      </c>
       <c r="E14" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H14" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="I14" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="J14" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="L14" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="M14" s="17" t="s">
         <v>46</v>
-      </c>
-      <c r="I14" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="J14" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="K14" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="L14" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="M14" s="17" t="s">
-        <v>47</v>
       </c>
       <c r="N14" s="18"/>
       <c r="O14" s="18"/>
       <c r="P14" s="18"/>
       <c r="Q14" s="18"/>
       <c r="R14" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="S14" s="18"/>
       <c r="T14" s="19"/>
@@ -3707,40 +3733,40 @@
     </row>
     <row r="15" spans="2:26" ht="15.75">
       <c r="B15" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C15" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" s="43" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="111" t="s">
+      <c r="E15" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="E15" s="16" t="s">
-        <v>121</v>
-      </c>
       <c r="F15" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H15" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="J15" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="I15" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="J15" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="K15" s="17" t="s">
-        <v>47</v>
-      </c>
       <c r="L15" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M15" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N15" s="18"/>
       <c r="O15" s="18"/>
@@ -3748,7 +3774,7 @@
       <c r="Q15" s="18"/>
       <c r="R15" s="18"/>
       <c r="S15" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="T15" s="19"/>
       <c r="U15" s="19">
@@ -3765,6 +3791,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F7:M7"/>
+    <mergeCell ref="N7:S7"/>
+    <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
     <mergeCell ref="D1:G1"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B6:B9"/>
@@ -3781,19 +3820,6 @@
     <mergeCell ref="W8:W9"/>
     <mergeCell ref="R8:R9"/>
     <mergeCell ref="T7:Z7"/>
-    <mergeCell ref="Z8:Z9"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:M7"/>
-    <mergeCell ref="N7:S7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3833,7 +3859,7 @@
     </row>
     <row r="3" spans="2:14">
       <c r="B3" s="66" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="66"/>
       <c r="D3" s="66"/>
@@ -3848,205 +3874,199 @@
     </row>
     <row r="4" spans="2:14">
       <c r="B4" s="67" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="74" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="D4" s="76" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="77" t="s">
+      <c r="E4" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="69" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="75"/>
-      <c r="I4" s="75"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="73"/>
       <c r="J4" s="70"/>
       <c r="K4" s="69" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L4" s="70"/>
     </row>
     <row r="5" spans="2:14" ht="14.65" thickBot="1">
       <c r="B5" s="68"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="78"/>
+      <c r="C5" s="75"/>
+      <c r="D5" s="77"/>
       <c r="E5" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F5" s="53" t="s">
         <v>122</v>
       </c>
-      <c r="F5" s="71" t="s">
-        <v>123</v>
-      </c>
-      <c r="G5" s="113"/>
-      <c r="H5" s="113"/>
-      <c r="I5" s="113"/>
-      <c r="J5" s="72"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="55"/>
       <c r="K5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="6" spans="2:14" ht="14.65" thickTop="1">
       <c r="B6" s="21">
         <v>9</v>
       </c>
-      <c r="C6" s="73" t="s">
-        <v>57</v>
+      <c r="C6" s="71" t="s">
+        <v>56</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="115" t="s">
-        <v>124</v>
-      </c>
-      <c r="F6" s="119" t="s">
-        <v>130</v>
-      </c>
-      <c r="G6" s="120"/>
-      <c r="H6" s="120"/>
-      <c r="I6" s="120"/>
-      <c r="J6" s="121"/>
-      <c r="K6" s="115" t="s">
-        <v>136</v>
-      </c>
-      <c r="L6" s="116" t="s">
-        <v>136</v>
-      </c>
-      <c r="M6" s="117"/>
+        <v>47</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="56" t="s">
+        <v>129</v>
+      </c>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="57"/>
+      <c r="J6" s="58"/>
+      <c r="K6" s="46" t="s">
+        <v>135</v>
+      </c>
+      <c r="L6" s="47" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="7" spans="2:14" ht="14.65" thickBot="1">
       <c r="B7" s="21">
         <v>10</v>
       </c>
-      <c r="C7" s="73"/>
+      <c r="C7" s="71"/>
       <c r="D7" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" s="116" t="s">
-        <v>125</v>
-      </c>
-      <c r="F7" s="122" t="s">
-        <v>131</v>
-      </c>
-      <c r="G7" s="123"/>
-      <c r="H7" s="123"/>
-      <c r="I7" s="123"/>
-      <c r="J7" s="124"/>
-      <c r="K7" s="116" t="s">
-        <v>137</v>
-      </c>
-      <c r="L7" s="116" t="s">
-        <v>137</v>
-      </c>
-      <c r="M7" s="117"/>
+        <v>57</v>
+      </c>
+      <c r="E7" s="47" t="s">
+        <v>124</v>
+      </c>
+      <c r="F7" s="59" t="s">
+        <v>130</v>
+      </c>
+      <c r="G7" s="60"/>
+      <c r="H7" s="60"/>
+      <c r="I7" s="60"/>
+      <c r="J7" s="61"/>
+      <c r="K7" s="47" t="s">
+        <v>136</v>
+      </c>
+      <c r="L7" s="47" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="8" spans="2:14" ht="14.65" thickTop="1">
       <c r="B8" s="21">
         <v>11</v>
       </c>
-      <c r="C8" s="73"/>
+      <c r="C8" s="71"/>
       <c r="D8" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="116" t="s">
-        <v>126</v>
-      </c>
-      <c r="F8" s="119" t="s">
-        <v>132</v>
-      </c>
-      <c r="G8" s="120"/>
-      <c r="H8" s="120"/>
-      <c r="I8" s="120"/>
-      <c r="J8" s="121"/>
-      <c r="K8" s="116" t="s">
-        <v>137</v>
-      </c>
-      <c r="L8" s="116" t="s">
-        <v>137</v>
-      </c>
-      <c r="M8" s="117"/>
+        <v>103</v>
+      </c>
+      <c r="E8" s="47" t="s">
+        <v>125</v>
+      </c>
+      <c r="F8" s="56" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" s="57"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="57"/>
+      <c r="J8" s="58"/>
+      <c r="K8" s="47" t="s">
+        <v>136</v>
+      </c>
+      <c r="L8" s="47" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="9" spans="2:14" ht="14.65" thickBot="1">
       <c r="B9" s="21">
         <v>12</v>
       </c>
-      <c r="C9" s="73"/>
+      <c r="C9" s="71"/>
       <c r="D9" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>126</v>
+      </c>
+      <c r="F9" s="59" t="s">
+        <v>132</v>
+      </c>
+      <c r="G9" s="60"/>
+      <c r="H9" s="60"/>
+      <c r="I9" s="60"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="47" t="s">
+        <v>137</v>
+      </c>
+      <c r="L9" s="47" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" ht="15" thickTop="1" thickBot="1">
+      <c r="B10" s="45">
+        <v>13</v>
+      </c>
+      <c r="C10" s="71"/>
+      <c r="D10" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="E9" s="116" t="s">
+      <c r="E10" t="s">
         <v>127</v>
       </c>
-      <c r="F9" s="122" t="s">
+      <c r="F10" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="123"/>
-      <c r="H9" s="123"/>
-      <c r="I9" s="123"/>
-      <c r="J9" s="124"/>
-      <c r="K9" s="116" t="s">
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="L9" s="116" t="s">
+      <c r="L10" s="47" t="s">
         <v>138</v>
       </c>
-      <c r="M9" s="117"/>
-    </row>
-    <row r="10" spans="2:14" ht="15" thickTop="1" thickBot="1">
-      <c r="B10" s="114">
-        <v>13</v>
-      </c>
-      <c r="C10" s="73"/>
-      <c r="D10" s="112" t="s">
-        <v>106</v>
-      </c>
-      <c r="E10" s="117" t="s">
-        <v>128</v>
-      </c>
-      <c r="F10" s="125" t="s">
-        <v>134</v>
-      </c>
-      <c r="G10" s="125"/>
-      <c r="H10" s="125"/>
-      <c r="I10" s="125"/>
-      <c r="J10" s="126"/>
-      <c r="K10" s="127" t="s">
-        <v>139</v>
-      </c>
-      <c r="L10" s="116" t="s">
-        <v>139</v>
-      </c>
-      <c r="M10" s="117"/>
     </row>
     <row r="11" spans="2:14" ht="15" thickTop="1" thickBot="1">
       <c r="B11" s="2">
         <v>14</v>
       </c>
-      <c r="C11" s="74"/>
+      <c r="C11" s="72"/>
       <c r="D11" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="E11" s="118" t="s">
-        <v>129</v>
-      </c>
-      <c r="F11" s="119" t="s">
-        <v>135</v>
-      </c>
-      <c r="G11" s="120"/>
-      <c r="H11" s="120"/>
-      <c r="I11" s="120"/>
-      <c r="J11" s="121"/>
-      <c r="K11" s="118" t="s">
-        <v>140</v>
-      </c>
-      <c r="L11" s="118" t="s">
-        <v>140</v>
-      </c>
-      <c r="M11" s="117"/>
+        <v>106</v>
+      </c>
+      <c r="E11" s="48" t="s">
+        <v>128</v>
+      </c>
+      <c r="F11" s="56" t="s">
+        <v>134</v>
+      </c>
+      <c r="G11" s="57"/>
+      <c r="H11" s="57"/>
+      <c r="I11" s="57"/>
+      <c r="J11" s="58"/>
+      <c r="K11" s="48" t="s">
+        <v>139</v>
+      </c>
+      <c r="L11" s="48" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="12" spans="2:14" ht="14.65" thickTop="1">
       <c r="B12" s="3"/>
@@ -4063,88 +4083,88 @@
     </row>
     <row r="13" spans="2:14" ht="14.65" thickBot="1">
       <c r="B13" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="K13" s="22"/>
+    </row>
+    <row r="14" spans="2:14" ht="15" thickTop="1" thickBot="1">
+      <c r="B14" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="K13" s="22"/>
-    </row>
-    <row r="14" spans="2:14" ht="15" thickTop="1" thickBot="1">
-      <c r="B14" s="55" t="s">
+      <c r="C14" s="52"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="78" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="47" t="s">
+      <c r="G14" s="79"/>
+      <c r="H14" s="51" t="s">
         <v>61</v>
       </c>
-      <c r="G14" s="48"/>
-      <c r="H14" s="55" t="s">
+      <c r="I14" s="52"/>
+      <c r="J14" s="52"/>
+      <c r="K14" s="52"/>
+      <c r="L14" s="88"/>
+      <c r="M14" s="93" t="s">
         <v>62</v>
       </c>
-      <c r="I14" s="56"/>
-      <c r="J14" s="56"/>
-      <c r="K14" s="56"/>
-      <c r="L14" s="57"/>
-      <c r="M14" s="61" t="s">
+      <c r="N14" s="94"/>
+    </row>
+    <row r="15" spans="2:14" ht="14.65" thickTop="1">
+      <c r="B15" s="92" t="s">
         <v>63</v>
       </c>
-      <c r="N14" s="62"/>
-    </row>
-    <row r="15" spans="2:14" ht="14.65" thickTop="1">
-      <c r="B15" s="39" t="s">
+      <c r="C15" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="C15" s="41" t="s">
+      <c r="D15" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="E15" s="96" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="43" t="s">
+      <c r="F15" s="81" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="45" t="s">
+      <c r="G15" s="80" t="s">
         <v>68</v>
       </c>
-      <c r="G15" s="49" t="s">
+      <c r="H15" s="82" t="s">
         <v>69</v>
       </c>
-      <c r="H15" s="51" t="s">
+      <c r="I15" s="84" t="s">
+        <v>63</v>
+      </c>
+      <c r="J15" s="84" t="s">
+        <v>64</v>
+      </c>
+      <c r="K15" s="86" t="s">
         <v>70</v>
       </c>
-      <c r="I15" s="41" t="s">
-        <v>64</v>
-      </c>
-      <c r="J15" s="41" t="s">
-        <v>65</v>
-      </c>
-      <c r="K15" s="53" t="s">
+      <c r="L15" s="89" t="s">
         <v>71</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="M15" s="91" t="s">
         <v>72</v>
       </c>
-      <c r="M15" s="60" t="s">
+      <c r="N15" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="N15" s="50" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="16" spans="2:14">
-      <c r="B16" s="40"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="52"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42"/>
-      <c r="K16" s="54"/>
-      <c r="L16" s="59"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="45"/>
+      <c r="B16" s="95"/>
+      <c r="C16" s="85"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="97"/>
+      <c r="F16" s="98"/>
+      <c r="G16" s="80"/>
+      <c r="H16" s="83"/>
+      <c r="I16" s="85"/>
+      <c r="J16" s="85"/>
+      <c r="K16" s="87"/>
+      <c r="L16" s="90"/>
+      <c r="M16" s="92"/>
+      <c r="N16" s="81"/>
     </row>
     <row r="17" spans="2:14">
       <c r="B17" s="26">
@@ -4163,10 +4183,10 @@
         <v>0</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I17" s="26">
         <f>SUM(J17:K17)</f>
@@ -4180,7 +4200,7 @@
       </c>
       <c r="L17" s="28"/>
       <c r="M17" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N17" s="29">
         <f>C17</f>
@@ -4189,6 +4209,28 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="M15:M16"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="C6:C11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="F5:J5"/>
     <mergeCell ref="F6:J6"/>
@@ -4197,30 +4239,8 @@
     <mergeCell ref="F9:J9"/>
     <mergeCell ref="F11:J11"/>
     <mergeCell ref="F10:I10"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="B3:L3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="C6:C11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
     <mergeCell ref="F14:G14"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="J15:J16"/>
     <mergeCell ref="H14:L14"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="M15:M16"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4417,15 +4437,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="301f98df-4edd-4096-94f8-2f8af3eee570">
@@ -4434,6 +4445,15 @@
     <TaxCatchAll xmlns="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4456,14 +4476,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EECFCB93-350B-4228-B7F4-DB12383611F2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2F5940-EC19-4D08-A8C2-FA31EF734077}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -4472,4 +4484,12 @@
     <ds:schemaRef ds:uri="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EECFCB93-350B-4228-B7F4-DB12383611F2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>